<commit_message>
Complete TLS2trees FOR-instance benchmark workflows
Add the exact manifest, source-row evaluation, development selection, retained prediction evidence, and guarded Barkla execution routes. Publish the neutral development-tuned result and add independent published-default and development diagnostic finalisation workflows.
</commit_message>
<xml_diff>
--- a/outputs/for_instance_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/for_instance_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="R22145fb569594b43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rff045f0d69124541"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="Rff179ee13d3241ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Ra632d449caf04fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="R69c5fc06ce644a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rc0118ad78b664cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="R898192c2487d4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Rdaed13b6db064782"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +45,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,6 +67,11 @@
         <x:fgColor rgb="FF1F7F9B"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -74,7 +79,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -130,6 +135,23 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -155,7 +177,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComparableResults" displayName="ComparableResults" ref="A4:Q9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComparableResults" displayName="ComparableResults" ref="A4:Q10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -172,7 +194,7 @@
     <x:tableColumn id="13" name="Micro recall"/>
     <x:tableColumn id="14" name="Micro F1"/>
     <x:tableColumn id="15" name="Δ mean F1 vs SAT published"/>
-    <x:tableColumn id="16" name="Evaluator"/>
+    <x:tableColumn id="16" name="Evaluation protocol"/>
     <x:tableColumn id="17" name="Retention"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -180,7 +202,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparableSiteResults" displayName="ComparableSiteResults" ref="A4:N29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparableSiteResults" displayName="ComparableSiteResults" ref="A4:N34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -202,7 +224,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ProtocolAlignment" displayName="ProtocolAlignment" ref="A4:J9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ProtocolAlignment" displayName="ProtocolAlignment" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -220,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComparableRetention" displayName="ComparableRetention" ref="A4:J9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ComparableRetention" displayName="ComparableRetention" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -447,34 +469,34 @@
     <x:col min="13" max="13" width="10" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="9.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="13.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="22.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="15" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="38" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>FOR-instance Comparable Held-out Results</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-      <x:c r="L1" s="3"/>
-      <x:c r="M1" s="3"/>
-      <x:c r="N1" s="3"/>
-      <x:c r="O1" s="3"/>
-      <x:c r="P1" s="3"/>
-      <x:c r="Q1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="25.5" customHeight="1">
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>FOR-instance Held-out Results</x:v>
+      </x:c>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="25"/>
+      <x:c r="D1" s="25"/>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="25"/>
+      <x:c r="H1" s="25"/>
+      <x:c r="I1" s="25"/>
+      <x:c r="J1" s="25"/>
+      <x:c r="K1" s="25"/>
+      <x:c r="L1" s="25"/>
+      <x:c r="M1" s="25"/>
+      <x:c r="N1" s="25"/>
+      <x:c r="O1" s="25"/>
+      <x:c r="P1" s="25"/>
+      <x:c r="Q1" s="25"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Five completed headline results: the same supplied 11-plot test split, 323 references, union mask, IoU threshold and one-to-one point-aligned evaluator.</x:v>
+        <x:v>Completed rows use the supplied test split and matching policy; the evaluation protocol column preserves scoring-domain differences.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -540,7 +562,7 @@
         <x:v>Δ mean F1 vs SAT published</x:v>
       </x:c>
       <x:c r="P4" s="11" t="str">
-        <x:v>Evaluator</x:v>
+        <x:v>Evaluation protocol</x:v>
       </x:c>
       <x:c r="Q4" s="11" t="str">
         <x:v>Retention</x:v>
@@ -813,6 +835,57 @@
         <x:v>for_instance_pointwise_v1</x:v>
       </x:c>
       <x:c r="Q9" s="12" t="str">
+        <x:v>retention_verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>external_training_only</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F10" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="G10" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H10" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I10" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="J10" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="K10" s="20" t="n">
+        <x:v>0.015022815022815023</x:v>
+      </x:c>
+      <x:c r="L10" s="20" t="n">
+        <x:v>0.07894736842105263</x:v>
+      </x:c>
+      <x:c r="M10" s="20" t="n">
+        <x:v>0.009287925696594427</x:v>
+      </x:c>
+      <x:c r="N10" s="20" t="n">
+        <x:v>0.01662049861495845</x:v>
+      </x:c>
+      <x:c r="O10" s="28"/>
+      <x:c r="P10" t="str">
+        <x:v>for_instance_pointwise_class3_ignore</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
     </x:row>
@@ -823,7 +896,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R057079016a6b4280"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916c274530134374"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -848,27 +921,30 @@
     <x:col min="14" max="14" width="9.4399995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="25" t="str">
         <x:v>FOR-instance Site Breakdown</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-      <x:c r="L1" s="3"/>
-      <x:c r="M1" s="3"/>
-      <x:c r="N1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="25"/>
+      <x:c r="D1" s="25"/>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="25"/>
+      <x:c r="H1" s="25"/>
+      <x:c r="I1" s="25"/>
+      <x:c r="J1" s="25"/>
+      <x:c r="K1" s="25"/>
+      <x:c r="L1" s="25"/>
+      <x:c r="M1" s="25"/>
+      <x:c r="N1" s="25"/>
+      <x:c r="O1" s="23"/>
+      <x:c r="P1" s="23"/>
+      <x:c r="Q1" s="23"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>All five headline variants are shown for CULS, NIBIO, RMIT, SCION and TUWIEN within the same held-out test comparison.</x:v>
+        <x:v>Site detail for completed held-out results; method, variant and protocol context are preserved in the source tables.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -883,6 +959,9 @@
       <x:c r="L2" s="7"/>
       <x:c r="M2" s="7"/>
       <x:c r="N2" s="7"/>
+      <x:c r="O2" s="23"/>
+      <x:c r="P2" s="23"/>
+      <x:c r="Q2" s="23"/>
     </x:row>
     <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -2026,6 +2105,226 @@
       </x:c>
       <x:c r="N29" s="15" t="n">
         <x:v>0.2891566265060241</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F30" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J30" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N30" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E31" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F31" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="H31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I31" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J31" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="K31" s="20" t="n">
+        <x:v>0.027541827541827543</x:v>
+      </x:c>
+      <x:c r="L31" s="20" t="n">
+        <x:v>0.08823529411764706</x:v>
+      </x:c>
+      <x:c r="M31" s="20" t="n">
+        <x:v>0.018633540372670808</x:v>
+      </x:c>
+      <x:c r="N31" s="20" t="n">
+        <x:v>0.03076923076923077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F32" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N32" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F33" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="K33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N33" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E34" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F34" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J34" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="K34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="20" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2035,7 +2334,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d3a9548a5343a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b000adb94c45a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2046,33 +2345,40 @@
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="8.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="8.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="23.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="23.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="42.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="25" t="str">
         <x:v>Protocol Alignment</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="25"/>
+      <x:c r="D1" s="25"/>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="25"/>
+      <x:c r="H1" s="25"/>
+      <x:c r="I1" s="25"/>
+      <x:c r="J1" s="25"/>
+      <x:c r="K1" s="23"/>
+      <x:c r="L1" s="23"/>
+      <x:c r="M1" s="23"/>
+      <x:c r="N1" s="23"/>
+      <x:c r="O1" s="23"/>
+      <x:c r="P1" s="23"/>
+      <x:c r="Q1" s="23"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Every headline row uses the official held-out subset and shared evaluator. Development-only diagnostics remain outside the headline table.</x:v>
+        <x:v>Protocol and scoring-domain differences remain explicit; rows are compared only within a compatible group.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2083,8 +2389,15 @@
       <x:c r="H2" s="7"/>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
-    </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+      <x:c r="K2" s="23"/>
+      <x:c r="L2" s="23"/>
+      <x:c r="M2" s="23"/>
+      <x:c r="N2" s="23"/>
+      <x:c r="O2" s="23"/>
+      <x:c r="P2" s="23"/>
+      <x:c r="Q2" s="23"/>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
         <x:v>Method</x:v>
       </x:c>
@@ -2116,23 +2429,23 @@
         <x:v>Interpretation</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="33" customHeight="1">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
         <x:v>Unsupervised parameterised</x:v>
       </x:c>
-      <x:c r="C5" s="12" t="str">
-        <x:v>Completed comparable</x:v>
-      </x:c>
-      <x:c r="D5" s="13" t="n">
+      <x:c r="C5" s="17" t="str">
+        <x:v>Legacy-v1 reported</x:v>
+      </x:c>
+      <x:c r="D5" s="26" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="n">
+      <x:c r="E5" s="26" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F5" s="14" t="n">
+      <x:c r="F5" s="27" t="n">
         <x:v>323</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
@@ -2148,23 +2461,23 @@
         <x:v>Deterministic non-learning method; no fine-tuned variant applies.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="33" customHeight="1">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
         <x:v>Published pretrained</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str">
-        <x:v>Completed comparable</x:v>
-      </x:c>
-      <x:c r="D6" s="13" t="n">
+      <x:c r="C6" s="17" t="str">
+        <x:v>Legacy-v1 reported</x:v>
+      </x:c>
+      <x:c r="D6" s="26" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E6" s="13" t="n">
+      <x:c r="E6" s="26" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F6" s="14" t="n">
+      <x:c r="F6" s="27" t="n">
         <x:v>323</x:v>
       </x:c>
       <x:c r="G6" s="17" t="str">
@@ -2180,23 +2493,23 @@
         <x:v>Published weights; no FOR-instance fine-tuning.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="33" customHeight="1">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
         <x:v>Fine-tuned on development data</x:v>
       </x:c>
-      <x:c r="C7" s="12" t="str">
-        <x:v>Completed comparable</x:v>
-      </x:c>
-      <x:c r="D7" s="13" t="n">
+      <x:c r="C7" s="17" t="str">
+        <x:v>Legacy-v1 reported</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E7" s="13" t="n">
+      <x:c r="E7" s="26" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F7" s="14" t="n">
+      <x:c r="F7" s="27" t="n">
         <x:v>323</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
@@ -2212,23 +2525,23 @@
         <x:v>Fine-tuned on development only; frozen checkpoint evaluated once.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="33" customHeight="1">
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>Published pretrained</x:v>
       </x:c>
-      <x:c r="C8" s="12" t="str">
-        <x:v>Completed comparable</x:v>
-      </x:c>
-      <x:c r="D8" s="13" t="n">
+      <x:c r="C8" s="17" t="str">
+        <x:v>Legacy-v1 reported</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E8" s="13" t="n">
+      <x:c r="E8" s="26" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F8" s="14" t="n">
+      <x:c r="F8" s="27" t="n">
         <x:v>323</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
@@ -2244,23 +2557,23 @@
         <x:v>Unchanged clean authors-released checkpoint; documented detection scope is trees above 10 m.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="33" customHeight="1">
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>Fine-tuned on development data</x:v>
       </x:c>
-      <x:c r="C9" s="12" t="str">
-        <x:v>Completed comparable</x:v>
-      </x:c>
-      <x:c r="D9" s="13" t="n">
+      <x:c r="C9" s="17" t="str">
+        <x:v>Legacy-v1 reported</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E9" s="13" t="n">
+      <x:c r="E9" s="26" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F9" s="14" t="n">
+      <x:c r="F9" s="27" t="n">
         <x:v>323</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
@@ -2274,6 +2587,38 @@
       </x:c>
       <x:c r="J9" s="17" t="str">
         <x:v>Fine-tuned on development only; frozen checkpoint evaluated once.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="32" hidden="0" customHeight="1">
+      <x:c r="A10" s="17" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Completed; separate scoring domain</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>for_instance_pointwise_class3_ignore</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str">
+        <x:v>Maximum-cardinality one-to-one</x:v>
+      </x:c>
+      <x:c r="I10" s="17" t="str">
+        <x:v>Frozen on development before held-out test</x:v>
+      </x:c>
+      <x:c r="J10" s="17" t="str">
+        <x:v>Leaf-on result excludes class-3 out-points; low accuracy indicates weak transfer from terrestrial to UAV laser scanning for this frozen pipeline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2283,7 +2628,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83413c1eb4d94efe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591296a148b04b90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2294,9 +2639,9 @@
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62.220001220703125" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="47.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="7.78000020980835" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="13.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16.110000610351562" hidden="0" customWidth="1"/>
@@ -2304,23 +2649,30 @@
     <x:col min="10" max="10" width="18.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Prediction Retention for Comparable Results</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="25.5" customHeight="1">
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>Prediction Retention</x:v>
+      </x:c>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="25"/>
+      <x:c r="D1" s="25"/>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="25"/>
+      <x:c r="H1" s="25"/>
+      <x:c r="I1" s="25"/>
+      <x:c r="J1" s="25"/>
+      <x:c r="K1" s="23"/>
+      <x:c r="L1" s="23"/>
+      <x:c r="M1" s="23"/>
+      <x:c r="N1" s="23"/>
+      <x:c r="O1" s="23"/>
+      <x:c r="P1" s="23"/>
+      <x:c r="Q1" s="23"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Primary prediction outputs remain outside Git and are retained so additional metrics can be computed without rerunning inference.</x:v>
+        <x:v>Primary outputs remain outside Git; every completed row names a retained, hash-verified prediction set.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2331,6 +2683,13 @@
       <x:c r="H2" s="7"/>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
+      <x:c r="K2" s="23"/>
+      <x:c r="L2" s="23"/>
+      <x:c r="M2" s="23"/>
+      <x:c r="N2" s="23"/>
+      <x:c r="O2" s="23"/>
+      <x:c r="P2" s="23"/>
+      <x:c r="Q2" s="23"/>
     </x:row>
     <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -2521,6 +2880,38 @@
         <x:v>barkla_run_scoped_retained</x:v>
       </x:c>
       <x:c r="J9" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Development tuned</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>tls2trees_for-instance_development_tuned_held_out_test_20260719_110219</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>22_source_row_aligned_npz_files_leaf_off_and_leaf_on</x:v>
+      </x:c>
+      <x:c r="F10" s="24" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G10" s="24" t="n">
+        <x:v>153398833</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>sha256_verified</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>barkla_run_scoped_retained</x:v>
+      </x:c>
+      <x:c r="J10" s="18" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2531,7 +2922,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4b8fa93a294c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd83ed8a50fb44258"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish TLS2trees published-default FOR-instance results
</commit_message>
<xml_diff>
--- a/outputs/for_instance_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/for_instance_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="R69c5fc06ce644a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rc0118ad78b664cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="R898192c2487d4b01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Rdaed13b6db064782"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="Ra78fdc0f688f4790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R123c8bab9e514432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="R412f314a5378426f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Rc4e75f32847f4753"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -177,7 +177,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComparableResults" displayName="ComparableResults" ref="A4:Q10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComparableResults" displayName="ComparableResults" ref="A4:Q11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -202,7 +202,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparableSiteResults" displayName="ComparableSiteResults" ref="A4:N34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparableSiteResults" displayName="ComparableSiteResults" ref="A4:N39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -224,7 +224,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ProtocolAlignment" displayName="ProtocolAlignment" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ProtocolAlignment" displayName="ProtocolAlignment" ref="A4:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ComparableRetention" displayName="ComparableRetention" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ComparableRetention" displayName="ComparableRetention" ref="A4:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -889,6 +889,57 @@
         <x:v>retention_verified</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>external_training_only</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F11" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="G11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J11" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="K11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11"/>
+      <x:c r="P11" t="str">
+        <x:v>for_instance_pointwise_class3_ignore</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>retention_verified</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
@@ -896,7 +947,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916c274530134374"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc707247da308454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2327,6 +2378,226 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F35" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J35" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E36" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="G36" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="K36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F37" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E38" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F38" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="K38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F39" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J39" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="K39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -2334,7 +2605,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b000adb94c45a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59dccddfd6564a18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2621,6 +2892,38 @@
         <x:v>Leaf-on result excludes class-3 out-points; low accuracy indicates weak transfer from terrestrial to UAV laser scanning for this frozen pipeline.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>Completed; separate scoring domain</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="str">
+        <x:v>for_instance_pointwise_class3_ignore</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="str">
+        <x:v>Maximum-cardinality one-to-one</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="str">
+        <x:v>No FOR-instance metric selection</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="str">
+        <x:v>Publication-derived parameters; leaf-on excludes class-3 out-points and was evaluated without FOR-instance metric selection.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -2628,7 +2931,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591296a148b04b90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cbe4c6217a14102"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2909,9 +3212,41 @@
         <x:v>sha256_verified</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>barkla_run_scoped_retained</x:v>
+        <x:v>run_scoped_retained</x:v>
       </x:c>
       <x:c r="J10" s="18" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>TLS2trees</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Published default</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>tls2trees_for-instance_published_default_held_out_test_20260721_122448</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>22_source_row_aligned_npz_files_leaf_off_and_leaf_on</x:v>
+      </x:c>
+      <x:c r="F11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G11" s="24" t="n">
+        <x:v>151789256</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>sha256_verified</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>run_scoped_retained</x:v>
+      </x:c>
+      <x:c r="J11" s="18" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2922,7 +3257,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd83ed8a50fb44258"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c1ad438f1cf4e89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>